<commit_message>
fix: PDF agent — use inline Part dicts instead of broken upload_file()
- genai.upload_file() does not accept file_data kwarg (TypeError)
- Switched to inline Part dicts: {mime_type, data} for PDFs/images
- Added data/ to .gitignore to prevent large DB files from being committed
- Added Econology Stage 2 Quote PDF to knowledge/

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lilamy_test_project/x1 client variation.xlsx
+++ b/lilamy_test_project/x1 client variation.xlsx
@@ -6,15 +6,17 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="920" firstSheet="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VO1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VO2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VO2" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VO1" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VO3" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internal VO Register" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VO6" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VO5" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internal VO Register" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Register'!$A$1:$M$38</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'Internal VO Register'!$A$1:$G$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'Register'!$A$1:$M$38</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'Internal VO Register'!$A$1:$G$21</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -1751,7 +1753,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="45" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="559">
+  <cellXfs count="560">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -3315,6 +3317,9 @@
     <xf numFmtId="4" fontId="14" fillId="0" borderId="4" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="5">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="4" fontId="15" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="108">
@@ -3921,7 +3926,9 @@
           <t>Date:</t>
         </is>
       </c>
-      <c r="G6" s="25" t="n"/>
+      <c r="G6" s="548" t="n">
+        <v>46187</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="89" t="inlineStr">
@@ -3948,7 +3955,7 @@
       </c>
       <c r="B8" s="90" t="inlineStr">
         <is>
-          <t>ass</t>
+          <t>ATRA</t>
         </is>
       </c>
       <c r="C8" s="91" t="n"/>
@@ -3987,7 +3994,7 @@
       <c r="A11" s="98" t="n"/>
       <c r="B11" s="99" t="inlineStr">
         <is>
-          <t xml:space="preserve">VO1 - east </t>
+          <t>VO2 - West</t>
         </is>
       </c>
       <c r="C11" s="100" t="n"/>
@@ -4050,11 +4057,11 @@
       </c>
       <c r="B14" s="329" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>BTEAR</t>
         </is>
       </c>
       <c r="C14" s="152" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D14" s="477" t="inlineStr">
         <is>
@@ -4062,14 +4069,14 @@
         </is>
       </c>
       <c r="E14" s="439" t="n">
-        <v>155</v>
+        <v>45555</v>
       </c>
       <c r="F14" s="478">
         <f>C14*E14</f>
         <v/>
       </c>
       <c r="G14" s="437" t="n">
-        <v>0</v>
+        <v>12000</v>
       </c>
       <c r="J14" s="438" t="n"/>
     </row>
@@ -4563,7 +4570,7 @@
         </is>
       </c>
       <c r="G6" s="548" t="n">
-        <v>46187</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="7">
@@ -4630,7 +4637,7 @@
       <c r="A11" s="98" t="n"/>
       <c r="B11" s="99" t="inlineStr">
         <is>
-          <t>VO2 - West</t>
+          <t xml:space="preserve">VO1 - east </t>
         </is>
       </c>
       <c r="C11" s="100" t="n"/>
@@ -4693,11 +4700,11 @@
       </c>
       <c r="B14" s="329" t="inlineStr">
         <is>
-          <t>BTEAR</t>
+          <t>132</t>
         </is>
       </c>
       <c r="C14" s="152" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D14" s="477" t="inlineStr">
         <is>
@@ -4705,14 +4712,14 @@
         </is>
       </c>
       <c r="E14" s="439" t="n">
-        <v>45555</v>
+        <v>155</v>
       </c>
       <c r="F14" s="478">
         <f>C14*E14</f>
         <v/>
       </c>
       <c r="G14" s="437" t="n">
-        <v>12000</v>
+        <v>0</v>
       </c>
       <c r="J14" s="438" t="n"/>
     </row>
@@ -5786,6 +5793,1368 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF92D050"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:J56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11.85546875" customWidth="1" style="22" min="1" max="1"/>
+    <col width="57.28515625" customWidth="1" style="23" min="2" max="2"/>
+    <col width="10.85546875" customWidth="1" min="3" max="4"/>
+    <col width="12.140625" customWidth="1" min="5" max="5"/>
+    <col width="13.5703125" customWidth="1" min="6" max="6"/>
+    <col width="13.5703125" customWidth="1" style="427" min="7" max="7"/>
+    <col width="10.5703125" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="25.7109375" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="18.75" customHeight="1">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="2" t="n"/>
+    </row>
+    <row r="4" ht="15.75" customHeight="1">
+      <c r="A4" s="353" t="inlineStr">
+        <is>
+          <t>CONTRACT VARIATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15.75" customHeight="1">
+      <c r="A5" s="4" t="n"/>
+      <c r="B5" s="24" t="n"/>
+      <c r="C5" s="353" t="n"/>
+      <c r="D5" s="353" t="n"/>
+      <c r="E5" s="353" t="n"/>
+      <c r="F5" s="353" t="n"/>
+      <c r="G5" s="366" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="89" t="inlineStr">
+        <is>
+          <t>PROJECT:</t>
+        </is>
+      </c>
+      <c r="B6" s="90" t="inlineStr">
+        <is>
+          <t>x1</t>
+        </is>
+      </c>
+      <c r="C6" s="91" t="n"/>
+      <c r="D6" s="92" t="n"/>
+      <c r="E6" s="92" t="n"/>
+      <c r="F6" s="92" t="inlineStr">
+        <is>
+          <t>Date:</t>
+        </is>
+      </c>
+      <c r="G6" s="548" t="n">
+        <v>46188</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="89" t="inlineStr">
+        <is>
+          <t>NAME:</t>
+        </is>
+      </c>
+      <c r="B7" s="90" t="inlineStr">
+        <is>
+          <t>Welink Construction</t>
+        </is>
+      </c>
+      <c r="C7" s="91" t="n"/>
+      <c r="D7" s="93" t="n"/>
+      <c r="E7" s="93" t="n"/>
+      <c r="F7" s="93" t="inlineStr"/>
+      <c r="G7" s="428" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="89" t="inlineStr">
+        <is>
+          <t>SITE ADDRESS:</t>
+        </is>
+      </c>
+      <c r="B8" s="90" t="inlineStr">
+        <is>
+          <t>ATRA</t>
+        </is>
+      </c>
+      <c r="C8" s="91" t="n"/>
+      <c r="D8" s="91" t="n"/>
+      <c r="E8" s="91" t="n"/>
+      <c r="F8" s="91" t="n"/>
+      <c r="G8" s="428" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="89" t="inlineStr">
+        <is>
+          <t>JOB No:</t>
+        </is>
+      </c>
+      <c r="B9" s="90" t="inlineStr">
+        <is>
+          <t>9876</t>
+        </is>
+      </c>
+      <c r="C9" s="95" t="n"/>
+      <c r="D9" s="95" t="n"/>
+      <c r="E9" s="95" t="n"/>
+      <c r="F9" s="95" t="n"/>
+      <c r="G9" s="428" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="96" t="n"/>
+      <c r="B10" s="97" t="n"/>
+      <c r="C10" s="95" t="n"/>
+      <c r="D10" s="95" t="n"/>
+      <c r="E10" s="95" t="n"/>
+      <c r="F10" s="95" t="n"/>
+      <c r="G10" s="428" t="n"/>
+    </row>
+    <row r="11" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A11" s="98" t="n"/>
+      <c r="B11" s="99" t="inlineStr">
+        <is>
+          <t>VO6 - Wet Fire Sprinkler Upgrade to Ground Floor</t>
+        </is>
+      </c>
+      <c r="C11" s="100" t="n"/>
+      <c r="D11" s="100" t="n"/>
+      <c r="E11" s="100" t="n"/>
+      <c r="F11" s="100" t="n"/>
+      <c r="G11" s="429" t="n"/>
+    </row>
+    <row r="12" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A12" s="102" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B12" s="430" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C12" s="369" t="n"/>
+      <c r="D12" s="369" t="n"/>
+      <c r="E12" s="370" t="n"/>
+      <c r="F12" s="103" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="G12" s="431" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="105" t="n"/>
+      <c r="B13" s="106" t="n"/>
+      <c r="C13" s="432" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="D13" s="432" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="E13" s="433" t="inlineStr">
+        <is>
+          <t>Rate ($)</t>
+        </is>
+      </c>
+      <c r="F13" s="434" t="n"/>
+      <c r="G13" s="435" t="n"/>
+      <c r="H13" s="436" t="n"/>
+      <c r="I13" s="436" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="107" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" s="329" t="inlineStr">
+        <is>
+          <t>100mm diameter fire sprinkler pipework</t>
+        </is>
+      </c>
+      <c r="C14" s="152" t="n">
+        <v>50</v>
+      </c>
+      <c r="D14" s="477" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E14" s="439" t="n">
+        <v>92</v>
+      </c>
+      <c r="F14" s="478">
+        <f>C14*E14</f>
+        <v/>
+      </c>
+      <c r="G14" s="437" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="438" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="107" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" s="82" t="inlineStr">
+        <is>
+          <t>New exposed sprinkler heads</t>
+        </is>
+      </c>
+      <c r="C15" s="152" t="n">
+        <v>12</v>
+      </c>
+      <c r="D15" s="477" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="E15" s="477" t="n">
+        <v>350</v>
+      </c>
+      <c r="F15" s="478">
+        <f>C15*E15</f>
+        <v/>
+      </c>
+      <c r="G15" s="437" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="479" t="n"/>
+      <c r="J15" s="438" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="82" t="inlineStr">
+        <is>
+          <t>Car stacker sprinkler heads</t>
+        </is>
+      </c>
+      <c r="C16" s="152" t="n">
+        <v>24</v>
+      </c>
+      <c r="D16" s="477" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="E16" s="477" t="n">
+        <v>280</v>
+      </c>
+      <c r="F16" s="478">
+        <f>C16*E16</f>
+        <v/>
+      </c>
+      <c r="G16" s="437" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="479" t="n"/>
+      <c r="J16" s="438" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="107" t="n">
+        <v>4</v>
+      </c>
+      <c r="B17" s="82" t="inlineStr">
+        <is>
+          <t>Pump exhaust reroute from basement to roof</t>
+        </is>
+      </c>
+      <c r="C17" s="152" t="n">
+        <v>30</v>
+      </c>
+      <c r="D17" s="477" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E17" s="439" t="n">
+        <v>200</v>
+      </c>
+      <c r="F17" s="478">
+        <f>C17*E17</f>
+        <v/>
+      </c>
+      <c r="G17" s="437" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="479" t="n"/>
+      <c r="J17" s="479" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="B18" s="82" t="inlineStr">
+        <is>
+          <t>Electrical attendance and builders works allowance</t>
+        </is>
+      </c>
+      <c r="C18" s="152" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="477" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="E18" s="439" t="n">
+        <v>5460</v>
+      </c>
+      <c r="F18" s="478">
+        <f>C18*E18</f>
+        <v/>
+      </c>
+      <c r="G18" s="437" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A19" s="109" t="n"/>
+      <c r="B19" s="85" t="n"/>
+      <c r="C19" s="86" t="n"/>
+      <c r="D19" s="442" t="n"/>
+      <c r="E19" s="443" t="n"/>
+      <c r="F19" s="444" t="n"/>
+      <c r="G19" s="445" t="n"/>
+    </row>
+    <row r="20" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A20" s="360" t="inlineStr">
+        <is>
+          <t>SUB TOTAL</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="8" t="n"/>
+      <c r="F20" s="446">
+        <f>SUM(F14:F19)</f>
+        <v/>
+      </c>
+      <c r="G20" s="447">
+        <f>SUM(G14:G19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="360" t="inlineStr">
+        <is>
+          <t>NETT VARIATION COST</t>
+        </is>
+      </c>
+      <c r="F21" s="448">
+        <f>F20-G20</f>
+        <v/>
+      </c>
+      <c r="G21" s="449" t="n"/>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="360" t="inlineStr">
+        <is>
+          <t>MARGIN AND OVERHEAD COSTS (10%)</t>
+        </is>
+      </c>
+      <c r="B22" s="360" t="n"/>
+      <c r="F22" s="450">
+        <f>F21*0.1</f>
+        <v/>
+      </c>
+      <c r="G22" s="451" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="360" t="inlineStr">
+        <is>
+          <t>VARIATION COST EXCLUDING GST</t>
+        </is>
+      </c>
+      <c r="B23" s="360" t="n"/>
+      <c r="F23" s="452">
+        <f>F21+F22</f>
+        <v/>
+      </c>
+      <c r="G23" s="453" t="n"/>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A24" s="360" t="inlineStr">
+        <is>
+          <t>GST</t>
+        </is>
+      </c>
+      <c r="B24" s="360" t="n"/>
+      <c r="F24" s="454">
+        <f>F23*0.1</f>
+        <v/>
+      </c>
+      <c r="G24" s="455" t="n"/>
+    </row>
+    <row r="25" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A25" s="360" t="inlineStr">
+        <is>
+          <t>TOTAL INCLUDING GST</t>
+        </is>
+      </c>
+      <c r="B25" s="360" t="n"/>
+      <c r="F25" s="456">
+        <f>F23+F24</f>
+        <v/>
+      </c>
+      <c r="G25" s="370" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="360" t="n"/>
+      <c r="C26" s="23" t="n"/>
+      <c r="D26" s="23" t="n"/>
+      <c r="E26" s="23" t="n"/>
+      <c r="F26" s="23" t="n"/>
+      <c r="G26" s="23" t="n"/>
+    </row>
+    <row r="27" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A27" s="360" t="n"/>
+      <c r="C27" s="457" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="34" t="n"/>
+      <c r="B28" s="9" t="n"/>
+      <c r="D28" s="458" t="n"/>
+      <c r="F28" s="459" t="inlineStr">
+        <is>
+          <t>Variation Raised By:</t>
+        </is>
+      </c>
+      <c r="G28" s="460" t="n"/>
+      <c r="I28" s="461" t="n"/>
+      <c r="J28" s="461" t="n"/>
+    </row>
+    <row r="29" ht="20.25" customHeight="1">
+      <c r="A29" s="34" t="n"/>
+      <c r="B29" s="9" t="n"/>
+      <c r="D29" s="462" t="n"/>
+      <c r="F29" s="463" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="G29" s="464" t="n"/>
+      <c r="I29" s="465" t="n"/>
+      <c r="J29" s="465" t="n"/>
+    </row>
+    <row r="30" ht="15" customHeight="1">
+      <c r="A30" s="34" t="n"/>
+      <c r="B30" s="9" t="n"/>
+      <c r="D30" s="462" t="n"/>
+      <c r="F30" s="466" t="n"/>
+      <c r="G30" s="467" t="n"/>
+      <c r="I30" s="465" t="n"/>
+      <c r="J30" s="465" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="360" t="inlineStr">
+        <is>
+          <t>ACCEPTED FOR AND ON BEHALF OF CLIENT:</t>
+        </is>
+      </c>
+      <c r="D31" s="458" t="n"/>
+      <c r="F31" s="468" t="inlineStr">
+        <is>
+          <t>Authorised By:</t>
+        </is>
+      </c>
+      <c r="G31" s="469" t="n"/>
+      <c r="I31" s="461" t="n"/>
+      <c r="J31" s="461" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="26" t="n"/>
+      <c r="B32" s="26" t="n"/>
+      <c r="D32" s="470" t="n"/>
+      <c r="F32" s="32" t="n"/>
+      <c r="G32" s="37" t="n"/>
+      <c r="I32" s="470" t="n"/>
+      <c r="J32" s="470" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="26" t="n"/>
+      <c r="B33" s="26" t="n"/>
+      <c r="D33" s="470" t="n"/>
+      <c r="F33" s="466" t="n"/>
+      <c r="G33" s="467" t="n"/>
+      <c r="I33" s="470" t="n"/>
+      <c r="J33" s="470" t="n"/>
+    </row>
+    <row r="34" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A34" s="361" t="n"/>
+      <c r="B34" s="403" t="n"/>
+      <c r="C34" s="471" t="n"/>
+      <c r="D34" s="471" t="n"/>
+      <c r="F34" s="472" t="n"/>
+      <c r="G34" s="473" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="34" t="n"/>
+      <c r="B35" s="9" t="n"/>
+      <c r="C35" s="471" t="n"/>
+      <c r="D35" s="471" t="n"/>
+      <c r="E35" s="470" t="n"/>
+      <c r="F35" s="470" t="n"/>
+      <c r="G35" s="470" t="n"/>
+    </row>
+    <row r="36">
+      <c r="C36" s="471" t="n"/>
+      <c r="D36" s="471" t="n"/>
+      <c r="E36" s="471" t="n"/>
+      <c r="F36" s="471" t="n"/>
+      <c r="G36" s="474" t="n"/>
+    </row>
+    <row r="37">
+      <c r="C37" s="471" t="n"/>
+      <c r="D37" s="471" t="n"/>
+      <c r="E37" s="471" t="n"/>
+      <c r="F37" s="471" t="n"/>
+      <c r="G37" s="474" t="n"/>
+    </row>
+    <row r="38">
+      <c r="C38" s="471" t="n"/>
+      <c r="D38" s="471" t="n"/>
+      <c r="E38" s="471" t="n"/>
+      <c r="F38" s="471" t="n"/>
+      <c r="G38" s="474" t="n"/>
+    </row>
+    <row r="39">
+      <c r="C39" s="471" t="n"/>
+      <c r="D39" s="471" t="n"/>
+      <c r="E39" s="471" t="n"/>
+      <c r="F39" s="471" t="n"/>
+      <c r="G39" s="474" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="17" t="n"/>
+      <c r="B40" s="18" t="n"/>
+      <c r="C40" s="6" t="n"/>
+      <c r="D40" s="6" t="n"/>
+      <c r="E40" s="6" t="n"/>
+      <c r="F40" s="6" t="n"/>
+      <c r="G40" s="475" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="17" t="n"/>
+      <c r="B41" s="18" t="n"/>
+      <c r="C41" s="6" t="n"/>
+      <c r="D41" s="6" t="n"/>
+      <c r="E41" s="6" t="n"/>
+      <c r="F41" s="6" t="n"/>
+      <c r="G41" s="475" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="17" t="n"/>
+      <c r="B42" s="18" t="n"/>
+      <c r="C42" s="6" t="n"/>
+      <c r="D42" s="6" t="n"/>
+      <c r="E42" s="6" t="n"/>
+      <c r="F42" s="6" t="n"/>
+      <c r="G42" s="475" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="n"/>
+      <c r="B43" s="18" t="n"/>
+      <c r="C43" s="6" t="n"/>
+      <c r="D43" s="6" t="n"/>
+      <c r="E43" s="6" t="n"/>
+      <c r="F43" s="6" t="n"/>
+      <c r="G43" s="475" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="17" t="n"/>
+      <c r="B44" s="18" t="n"/>
+      <c r="C44" s="6" t="n"/>
+      <c r="D44" s="6" t="n"/>
+      <c r="E44" s="6" t="n"/>
+      <c r="F44" s="6" t="n"/>
+      <c r="G44" s="475" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="17" t="n"/>
+      <c r="B45" s="18" t="n"/>
+      <c r="C45" s="6" t="n"/>
+      <c r="D45" s="6" t="n"/>
+      <c r="E45" s="6" t="n"/>
+      <c r="F45" s="6" t="n"/>
+      <c r="G45" s="475" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="19" t="n"/>
+      <c r="B46" s="20" t="n"/>
+      <c r="C46" s="6" t="n"/>
+      <c r="D46" s="6" t="n"/>
+      <c r="E46" s="6" t="n"/>
+      <c r="F46" s="6" t="n"/>
+      <c r="G46" s="476" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="n"/>
+      <c r="B47" s="18" t="n"/>
+      <c r="C47" s="6" t="n"/>
+      <c r="D47" s="6" t="n"/>
+      <c r="E47" s="6" t="n"/>
+      <c r="F47" s="6" t="n"/>
+      <c r="G47" s="475" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="19" t="n"/>
+      <c r="B48" s="20" t="n"/>
+      <c r="C48" s="6" t="n"/>
+      <c r="D48" s="6" t="n"/>
+      <c r="E48" s="6" t="n"/>
+      <c r="F48" s="6" t="n"/>
+      <c r="G48" s="476" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="n"/>
+      <c r="B49" s="18" t="n"/>
+      <c r="C49" s="6" t="n"/>
+      <c r="D49" s="6" t="n"/>
+      <c r="E49" s="6" t="n"/>
+      <c r="F49" s="6" t="n"/>
+      <c r="G49" s="475" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="19" t="n"/>
+      <c r="B50" s="20" t="n"/>
+      <c r="C50" s="6" t="n"/>
+      <c r="D50" s="6" t="n"/>
+      <c r="E50" s="6" t="n"/>
+      <c r="F50" s="6" t="n"/>
+      <c r="G50" s="476" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="n"/>
+      <c r="B51" s="18" t="n"/>
+      <c r="C51" s="6" t="n"/>
+      <c r="D51" s="6" t="n"/>
+      <c r="E51" s="6" t="n"/>
+      <c r="F51" s="6" t="n"/>
+      <c r="G51" s="475" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="n"/>
+      <c r="B52" s="18" t="n"/>
+      <c r="C52" s="6" t="n"/>
+      <c r="D52" s="6" t="n"/>
+      <c r="E52" s="6" t="n"/>
+      <c r="F52" s="6" t="n"/>
+      <c r="G52" s="475" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="n"/>
+      <c r="B53" s="18" t="n"/>
+      <c r="C53" s="6" t="n"/>
+      <c r="D53" s="6" t="n"/>
+      <c r="E53" s="6" t="n"/>
+      <c r="F53" s="6" t="n"/>
+      <c r="G53" s="475" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="n"/>
+      <c r="B54" s="18" t="n"/>
+      <c r="C54" s="6" t="n"/>
+      <c r="D54" s="6" t="n"/>
+      <c r="E54" s="6" t="n"/>
+      <c r="F54" s="6" t="n"/>
+      <c r="G54" s="475" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="n"/>
+      <c r="B55" s="18" t="n"/>
+      <c r="C55" s="6" t="n"/>
+      <c r="D55" s="6" t="n"/>
+      <c r="E55" s="6" t="n"/>
+      <c r="F55" s="6" t="n"/>
+      <c r="G55" s="475" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="17" t="n"/>
+      <c r="B56" s="18" t="n"/>
+      <c r="C56" s="6" t="n"/>
+      <c r="D56" s="6" t="n"/>
+      <c r="E56" s="6" t="n"/>
+      <c r="F56" s="6" t="n"/>
+      <c r="G56" s="475" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A34:B34"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="67"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF92D050"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:J56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11.85546875" customWidth="1" style="22" min="1" max="1"/>
+    <col width="57.28515625" customWidth="1" style="23" min="2" max="2"/>
+    <col width="10.85546875" customWidth="1" min="3" max="4"/>
+    <col width="12.140625" customWidth="1" min="5" max="5"/>
+    <col width="13.5703125" customWidth="1" min="6" max="6"/>
+    <col width="13.5703125" customWidth="1" style="427" min="7" max="7"/>
+    <col width="10.5703125" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="25.7109375" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="18.75" customHeight="1">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="2" t="n"/>
+    </row>
+    <row r="4" ht="15.75" customHeight="1">
+      <c r="A4" s="353" t="inlineStr">
+        <is>
+          <t>CONTRACT VARIATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15.75" customHeight="1">
+      <c r="A5" s="4" t="n"/>
+      <c r="B5" s="24" t="n"/>
+      <c r="C5" s="353" t="n"/>
+      <c r="D5" s="353" t="n"/>
+      <c r="E5" s="353" t="n"/>
+      <c r="F5" s="353" t="n"/>
+      <c r="G5" s="366" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="89" t="inlineStr">
+        <is>
+          <t>PROJECT:</t>
+        </is>
+      </c>
+      <c r="B6" s="90" t="inlineStr">
+        <is>
+          <t>x1</t>
+        </is>
+      </c>
+      <c r="C6" s="91" t="n"/>
+      <c r="D6" s="92" t="n"/>
+      <c r="E6" s="92" t="n"/>
+      <c r="F6" s="92" t="inlineStr">
+        <is>
+          <t>Date:</t>
+        </is>
+      </c>
+      <c r="G6" s="548" t="n">
+        <v>46188</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="89" t="inlineStr">
+        <is>
+          <t>NAME:</t>
+        </is>
+      </c>
+      <c r="B7" s="90" t="inlineStr">
+        <is>
+          <t>Welink Construction</t>
+        </is>
+      </c>
+      <c r="C7" s="91" t="n"/>
+      <c r="D7" s="93" t="n"/>
+      <c r="E7" s="93" t="n"/>
+      <c r="F7" s="93" t="inlineStr"/>
+      <c r="G7" s="428" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="89" t="inlineStr">
+        <is>
+          <t>SITE ADDRESS:</t>
+        </is>
+      </c>
+      <c r="B8" s="90" t="inlineStr">
+        <is>
+          <t>ATRA</t>
+        </is>
+      </c>
+      <c r="C8" s="91" t="n"/>
+      <c r="D8" s="91" t="n"/>
+      <c r="E8" s="91" t="n"/>
+      <c r="F8" s="91" t="n"/>
+      <c r="G8" s="428" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="89" t="inlineStr">
+        <is>
+          <t>JOB No:</t>
+        </is>
+      </c>
+      <c r="B9" s="90" t="inlineStr">
+        <is>
+          <t>9876</t>
+        </is>
+      </c>
+      <c r="C9" s="95" t="n"/>
+      <c r="D9" s="95" t="n"/>
+      <c r="E9" s="95" t="n"/>
+      <c r="F9" s="95" t="n"/>
+      <c r="G9" s="428" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="96" t="n"/>
+      <c r="B10" s="97" t="n"/>
+      <c r="C10" s="95" t="n"/>
+      <c r="D10" s="95" t="n"/>
+      <c r="E10" s="95" t="n"/>
+      <c r="F10" s="95" t="n"/>
+      <c r="G10" s="428" t="n"/>
+    </row>
+    <row r="11" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A11" s="98" t="n"/>
+      <c r="B11" s="99" t="inlineStr">
+        <is>
+          <t>VO5 - asdasdasdasd</t>
+        </is>
+      </c>
+      <c r="C11" s="100" t="n"/>
+      <c r="D11" s="100" t="n"/>
+      <c r="E11" s="100" t="n"/>
+      <c r="F11" s="100" t="n"/>
+      <c r="G11" s="429" t="n"/>
+    </row>
+    <row r="12" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A12" s="102" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B12" s="430" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C12" s="369" t="n"/>
+      <c r="D12" s="369" t="n"/>
+      <c r="E12" s="370" t="n"/>
+      <c r="F12" s="103" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="G12" s="431" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="105" t="n"/>
+      <c r="B13" s="106" t="n"/>
+      <c r="C13" s="432" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="D13" s="432" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="E13" s="433" t="inlineStr">
+        <is>
+          <t>Rate ($)</t>
+        </is>
+      </c>
+      <c r="F13" s="434" t="n"/>
+      <c r="G13" s="435" t="n"/>
+      <c r="H13" s="436" t="n"/>
+      <c r="I13" s="436" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="107" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" s="329" t="inlineStr">
+        <is>
+          <t>123123123</t>
+        </is>
+      </c>
+      <c r="C14" s="152" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="477" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="E14" s="439" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F14" s="478">
+        <f>C14*E14</f>
+        <v/>
+      </c>
+      <c r="G14" s="437" t="n">
+        <v>2000</v>
+      </c>
+      <c r="J14" s="438" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="107" t="n"/>
+      <c r="B15" s="82" t="n"/>
+      <c r="C15" s="152" t="n"/>
+      <c r="D15" s="477" t="n"/>
+      <c r="E15" s="477" t="n"/>
+      <c r="F15" s="478" t="n"/>
+      <c r="G15" s="437" t="n"/>
+      <c r="I15" s="479" t="n"/>
+      <c r="J15" s="438" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="107" t="n"/>
+      <c r="B16" s="82" t="n"/>
+      <c r="C16" s="152" t="n"/>
+      <c r="D16" s="477" t="n"/>
+      <c r="E16" s="477" t="n"/>
+      <c r="F16" s="478" t="n"/>
+      <c r="G16" s="437" t="n"/>
+      <c r="I16" s="479" t="n"/>
+      <c r="J16" s="438" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="107" t="n"/>
+      <c r="B17" s="82" t="n"/>
+      <c r="C17" s="152" t="n"/>
+      <c r="D17" s="477" t="n"/>
+      <c r="E17" s="439" t="n"/>
+      <c r="F17" s="478" t="n"/>
+      <c r="G17" s="437" t="n"/>
+      <c r="I17" s="479" t="n"/>
+      <c r="J17" s="479" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="107" t="n"/>
+      <c r="B18" s="82" t="n"/>
+      <c r="C18" s="152" t="n"/>
+      <c r="D18" s="477" t="n"/>
+      <c r="E18" s="439" t="n"/>
+      <c r="F18" s="478" t="n"/>
+      <c r="G18" s="437" t="n"/>
+    </row>
+    <row r="19" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A19" s="109" t="n"/>
+      <c r="B19" s="85" t="n"/>
+      <c r="C19" s="86" t="n"/>
+      <c r="D19" s="442" t="n"/>
+      <c r="E19" s="443" t="n"/>
+      <c r="F19" s="444" t="n"/>
+      <c r="G19" s="445" t="n"/>
+    </row>
+    <row r="20" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A20" s="360" t="inlineStr">
+        <is>
+          <t>SUB TOTAL</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="8" t="n"/>
+      <c r="F20" s="446">
+        <f>SUM(F14:F19)</f>
+        <v/>
+      </c>
+      <c r="G20" s="447">
+        <f>SUM(G14:G19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="360" t="inlineStr">
+        <is>
+          <t>NETT VARIATION COST</t>
+        </is>
+      </c>
+      <c r="F21" s="448">
+        <f>F20-G20</f>
+        <v/>
+      </c>
+      <c r="G21" s="449" t="n"/>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="360" t="inlineStr">
+        <is>
+          <t>MARGIN AND OVERHEAD COSTS (10%)</t>
+        </is>
+      </c>
+      <c r="B22" s="360" t="n"/>
+      <c r="F22" s="450">
+        <f>F21*0.1</f>
+        <v/>
+      </c>
+      <c r="G22" s="451" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="360" t="inlineStr">
+        <is>
+          <t>VARIATION COST EXCLUDING GST</t>
+        </is>
+      </c>
+      <c r="B23" s="360" t="n"/>
+      <c r="F23" s="452">
+        <f>F21+F22</f>
+        <v/>
+      </c>
+      <c r="G23" s="453" t="n"/>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A24" s="360" t="inlineStr">
+        <is>
+          <t>GST</t>
+        </is>
+      </c>
+      <c r="B24" s="360" t="n"/>
+      <c r="F24" s="454">
+        <f>F23*0.1</f>
+        <v/>
+      </c>
+      <c r="G24" s="455" t="n"/>
+    </row>
+    <row r="25" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A25" s="360" t="inlineStr">
+        <is>
+          <t>TOTAL INCLUDING GST</t>
+        </is>
+      </c>
+      <c r="B25" s="360" t="n"/>
+      <c r="F25" s="456">
+        <f>F23+F24</f>
+        <v/>
+      </c>
+      <c r="G25" s="370" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="360" t="n"/>
+      <c r="C26" s="23" t="n"/>
+      <c r="D26" s="23" t="n"/>
+      <c r="E26" s="23" t="n"/>
+      <c r="F26" s="23" t="n"/>
+      <c r="G26" s="23" t="n"/>
+    </row>
+    <row r="27" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A27" s="360" t="n"/>
+      <c r="C27" s="457" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="34" t="n"/>
+      <c r="B28" s="9" t="n"/>
+      <c r="D28" s="458" t="n"/>
+      <c r="F28" s="459" t="inlineStr">
+        <is>
+          <t>Variation Raised By:</t>
+        </is>
+      </c>
+      <c r="G28" s="460" t="n"/>
+      <c r="I28" s="461" t="n"/>
+      <c r="J28" s="461" t="n"/>
+    </row>
+    <row r="29" ht="20.25" customHeight="1">
+      <c r="A29" s="34" t="n"/>
+      <c r="B29" s="9" t="n"/>
+      <c r="D29" s="462" t="n"/>
+      <c r="F29" s="463" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="G29" s="464" t="n"/>
+      <c r="I29" s="465" t="n"/>
+      <c r="J29" s="465" t="n"/>
+    </row>
+    <row r="30" ht="15" customHeight="1">
+      <c r="A30" s="34" t="n"/>
+      <c r="B30" s="9" t="n"/>
+      <c r="D30" s="462" t="n"/>
+      <c r="F30" s="466" t="n"/>
+      <c r="G30" s="467" t="n"/>
+      <c r="I30" s="465" t="n"/>
+      <c r="J30" s="465" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="360" t="inlineStr">
+        <is>
+          <t>ACCEPTED FOR AND ON BEHALF OF CLIENT:</t>
+        </is>
+      </c>
+      <c r="D31" s="458" t="n"/>
+      <c r="F31" s="468" t="inlineStr">
+        <is>
+          <t>Authorised By:</t>
+        </is>
+      </c>
+      <c r="G31" s="469" t="n"/>
+      <c r="I31" s="461" t="n"/>
+      <c r="J31" s="461" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="26" t="n"/>
+      <c r="B32" s="26" t="n"/>
+      <c r="D32" s="470" t="n"/>
+      <c r="F32" s="32" t="n"/>
+      <c r="G32" s="37" t="n"/>
+      <c r="I32" s="470" t="n"/>
+      <c r="J32" s="470" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="26" t="n"/>
+      <c r="B33" s="26" t="n"/>
+      <c r="D33" s="470" t="n"/>
+      <c r="F33" s="466" t="n"/>
+      <c r="G33" s="467" t="n"/>
+      <c r="I33" s="470" t="n"/>
+      <c r="J33" s="470" t="n"/>
+    </row>
+    <row r="34" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A34" s="361" t="n"/>
+      <c r="B34" s="403" t="n"/>
+      <c r="C34" s="471" t="n"/>
+      <c r="D34" s="471" t="n"/>
+      <c r="F34" s="472" t="n"/>
+      <c r="G34" s="473" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="34" t="n"/>
+      <c r="B35" s="9" t="n"/>
+      <c r="C35" s="471" t="n"/>
+      <c r="D35" s="471" t="n"/>
+      <c r="E35" s="470" t="n"/>
+      <c r="F35" s="470" t="n"/>
+      <c r="G35" s="470" t="n"/>
+    </row>
+    <row r="36">
+      <c r="C36" s="471" t="n"/>
+      <c r="D36" s="471" t="n"/>
+      <c r="E36" s="471" t="n"/>
+      <c r="F36" s="471" t="n"/>
+      <c r="G36" s="474" t="n"/>
+    </row>
+    <row r="37">
+      <c r="C37" s="471" t="n"/>
+      <c r="D37" s="471" t="n"/>
+      <c r="E37" s="471" t="n"/>
+      <c r="F37" s="471" t="n"/>
+      <c r="G37" s="474" t="n"/>
+    </row>
+    <row r="38">
+      <c r="C38" s="471" t="n"/>
+      <c r="D38" s="471" t="n"/>
+      <c r="E38" s="471" t="n"/>
+      <c r="F38" s="471" t="n"/>
+      <c r="G38" s="474" t="n"/>
+    </row>
+    <row r="39">
+      <c r="C39" s="471" t="n"/>
+      <c r="D39" s="471" t="n"/>
+      <c r="E39" s="471" t="n"/>
+      <c r="F39" s="471" t="n"/>
+      <c r="G39" s="474" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="17" t="n"/>
+      <c r="B40" s="18" t="n"/>
+      <c r="C40" s="6" t="n"/>
+      <c r="D40" s="6" t="n"/>
+      <c r="E40" s="6" t="n"/>
+      <c r="F40" s="6" t="n"/>
+      <c r="G40" s="475" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="17" t="n"/>
+      <c r="B41" s="18" t="n"/>
+      <c r="C41" s="6" t="n"/>
+      <c r="D41" s="6" t="n"/>
+      <c r="E41" s="6" t="n"/>
+      <c r="F41" s="6" t="n"/>
+      <c r="G41" s="475" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="17" t="n"/>
+      <c r="B42" s="18" t="n"/>
+      <c r="C42" s="6" t="n"/>
+      <c r="D42" s="6" t="n"/>
+      <c r="E42" s="6" t="n"/>
+      <c r="F42" s="6" t="n"/>
+      <c r="G42" s="475" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="n"/>
+      <c r="B43" s="18" t="n"/>
+      <c r="C43" s="6" t="n"/>
+      <c r="D43" s="6" t="n"/>
+      <c r="E43" s="6" t="n"/>
+      <c r="F43" s="6" t="n"/>
+      <c r="G43" s="475" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="17" t="n"/>
+      <c r="B44" s="18" t="n"/>
+      <c r="C44" s="6" t="n"/>
+      <c r="D44" s="6" t="n"/>
+      <c r="E44" s="6" t="n"/>
+      <c r="F44" s="6" t="n"/>
+      <c r="G44" s="475" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="17" t="n"/>
+      <c r="B45" s="18" t="n"/>
+      <c r="C45" s="6" t="n"/>
+      <c r="D45" s="6" t="n"/>
+      <c r="E45" s="6" t="n"/>
+      <c r="F45" s="6" t="n"/>
+      <c r="G45" s="475" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="19" t="n"/>
+      <c r="B46" s="20" t="n"/>
+      <c r="C46" s="6" t="n"/>
+      <c r="D46" s="6" t="n"/>
+      <c r="E46" s="6" t="n"/>
+      <c r="F46" s="6" t="n"/>
+      <c r="G46" s="476" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="n"/>
+      <c r="B47" s="18" t="n"/>
+      <c r="C47" s="6" t="n"/>
+      <c r="D47" s="6" t="n"/>
+      <c r="E47" s="6" t="n"/>
+      <c r="F47" s="6" t="n"/>
+      <c r="G47" s="475" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="19" t="n"/>
+      <c r="B48" s="20" t="n"/>
+      <c r="C48" s="6" t="n"/>
+      <c r="D48" s="6" t="n"/>
+      <c r="E48" s="6" t="n"/>
+      <c r="F48" s="6" t="n"/>
+      <c r="G48" s="476" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="n"/>
+      <c r="B49" s="18" t="n"/>
+      <c r="C49" s="6" t="n"/>
+      <c r="D49" s="6" t="n"/>
+      <c r="E49" s="6" t="n"/>
+      <c r="F49" s="6" t="n"/>
+      <c r="G49" s="475" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="19" t="n"/>
+      <c r="B50" s="20" t="n"/>
+      <c r="C50" s="6" t="n"/>
+      <c r="D50" s="6" t="n"/>
+      <c r="E50" s="6" t="n"/>
+      <c r="F50" s="6" t="n"/>
+      <c r="G50" s="476" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="n"/>
+      <c r="B51" s="18" t="n"/>
+      <c r="C51" s="6" t="n"/>
+      <c r="D51" s="6" t="n"/>
+      <c r="E51" s="6" t="n"/>
+      <c r="F51" s="6" t="n"/>
+      <c r="G51" s="475" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="n"/>
+      <c r="B52" s="18" t="n"/>
+      <c r="C52" s="6" t="n"/>
+      <c r="D52" s="6" t="n"/>
+      <c r="E52" s="6" t="n"/>
+      <c r="F52" s="6" t="n"/>
+      <c r="G52" s="475" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="n"/>
+      <c r="B53" s="18" t="n"/>
+      <c r="C53" s="6" t="n"/>
+      <c r="D53" s="6" t="n"/>
+      <c r="E53" s="6" t="n"/>
+      <c r="F53" s="6" t="n"/>
+      <c r="G53" s="475" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="n"/>
+      <c r="B54" s="18" t="n"/>
+      <c r="C54" s="6" t="n"/>
+      <c r="D54" s="6" t="n"/>
+      <c r="E54" s="6" t="n"/>
+      <c r="F54" s="6" t="n"/>
+      <c r="G54" s="475" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="n"/>
+      <c r="B55" s="18" t="n"/>
+      <c r="C55" s="6" t="n"/>
+      <c r="D55" s="6" t="n"/>
+      <c r="E55" s="6" t="n"/>
+      <c r="F55" s="6" t="n"/>
+      <c r="G55" s="475" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="17" t="n"/>
+      <c r="B56" s="18" t="n"/>
+      <c r="C56" s="6" t="n"/>
+      <c r="D56" s="6" t="n"/>
+      <c r="E56" s="6" t="n"/>
+      <c r="F56" s="6" t="n"/>
+      <c r="G56" s="475" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A34:B34"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="67"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7018,25 +8387,29 @@
     </row>
     <row r="13" ht="28.9" customHeight="1">
       <c r="A13" s="60" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B13" s="333" t="inlineStr">
         <is>
-          <t xml:space="preserve">VO1 - east </t>
-        </is>
-      </c>
-      <c r="C13" s="503" t="n"/>
+          <t>VO2 - West</t>
+        </is>
+      </c>
+      <c r="C13" s="503" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
       <c r="D13" s="504" t="n">
-        <v>1687.95</v>
+        <v>40601.55</v>
       </c>
       <c r="E13" s="505" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="506" t="n">
-        <v>687.95</v>
+        <v>15121.55</v>
       </c>
       <c r="G13" s="507" t="n">
-        <v>1000</v>
+        <v>40000</v>
       </c>
       <c r="H13" s="508" t="n"/>
       <c r="I13" s="508" t="n"/>
@@ -7056,29 +8429,29 @@
     </row>
     <row r="14" ht="28.9" customHeight="1">
       <c r="A14" s="60" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B14" s="333" t="inlineStr">
         <is>
-          <t>VO2 - West</t>
+          <t xml:space="preserve">VO1 - east </t>
         </is>
       </c>
       <c r="C14" s="503" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="D14" s="504" t="n">
-        <v>40601.55</v>
+        <v>1687.95</v>
       </c>
       <c r="E14" s="505" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="506" t="n">
-        <v>15121.55</v>
+        <v>687.95</v>
       </c>
       <c r="G14" s="507" t="n">
-        <v>40000</v>
+        <v>1000</v>
       </c>
       <c r="H14" s="509" t="n"/>
       <c r="I14" s="509" t="n"/>
@@ -7102,19 +8475,19 @@
       </c>
       <c r="B15" s="333" t="inlineStr">
         <is>
-          <t>VO3 - BEEASt</t>
+          <t>VO5 - asdasdasdasd</t>
         </is>
       </c>
       <c r="C15" s="503" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="D15" s="504" t="n">
-        <v>21780</v>
+        <v>20570</v>
       </c>
       <c r="E15" s="505" t="n">
-        <v>21780</v>
+        <v>20570</v>
       </c>
       <c r="F15" s="506" t="n">
         <v>0</v>
@@ -7139,18 +8512,44 @@
       <c r="N15" s="59" t="n"/>
     </row>
     <row r="16" ht="28.9" customHeight="1">
-      <c r="A16" s="60" t="n"/>
-      <c r="B16" s="334" t="n"/>
-      <c r="C16" s="503" t="n"/>
-      <c r="D16" s="504" t="n"/>
-      <c r="E16" s="505" t="n"/>
-      <c r="F16" s="506" t="n"/>
-      <c r="G16" s="507" t="n"/>
+      <c r="A16" s="60" t="n">
+        <v>6</v>
+      </c>
+      <c r="B16" s="334" t="inlineStr">
+        <is>
+          <t>VO6 - Wet Fire Sprinkler Upgrade to Ground Floor</t>
+        </is>
+      </c>
+      <c r="C16" s="503" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="D16" s="504" t="n">
+        <v>32645.8</v>
+      </c>
+      <c r="E16" s="505" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="506" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="507" t="n">
+        <v>36154.8</v>
+      </c>
       <c r="H16" s="509" t="n"/>
       <c r="I16" s="509" t="n"/>
       <c r="J16" s="76" t="n"/>
-      <c r="K16" s="77" t="n"/>
-      <c r="L16" s="146" t="n"/>
+      <c r="K16" s="549" t="inlineStr">
+        <is>
+          <t>Approved for Signing</t>
+        </is>
+      </c>
+      <c r="L16" s="146" t="inlineStr">
+        <is>
+          <t>Head Contract VO</t>
+        </is>
+      </c>
       <c r="M16" s="66" t="n"/>
       <c r="N16" s="59" t="n"/>
     </row>
@@ -7499,16 +8898,16 @@
       </c>
       <c r="C38" s="120" t="n"/>
       <c r="D38" s="518" t="n">
-        <v>64069.5</v>
+        <v>95505.3</v>
       </c>
       <c r="E38" s="519" t="n">
-        <v>21780</v>
+        <v>20570</v>
       </c>
       <c r="F38" s="520" t="n">
         <v>15809.5</v>
       </c>
       <c r="G38" s="521" t="n">
-        <v>41000</v>
+        <v>77154.8</v>
       </c>
       <c r="H38" s="522">
         <f>SUM(H13:H37)</f>
@@ -7610,7 +9009,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8644,46 +10043,74 @@
       <c r="G6" s="184" t="n"/>
     </row>
     <row r="7" ht="28.9" customHeight="1">
-      <c r="A7" s="60" t="n"/>
+      <c r="A7" s="60" t="n">
+        <v>4</v>
+      </c>
       <c r="B7" s="331" t="inlineStr">
         <is>
-          <t>TOTALS</t>
-        </is>
-      </c>
-      <c r="C7" s="539">
-        <f>SUM(C4:C6)</f>
-        <v/>
-      </c>
-      <c r="D7" s="516">
-        <f>SUM(D4:D6)</f>
-        <v/>
-      </c>
-      <c r="E7" s="540">
-        <f>SUM(E4:E6)</f>
-        <v/>
-      </c>
-      <c r="F7" s="214">
-        <f>SUM(F4:F6)</f>
-        <v/>
+          <t>VO5 - asdasdasdasd</t>
+        </is>
+      </c>
+      <c r="C7" s="554" t="n">
+        <v>20570</v>
+      </c>
+      <c r="D7" s="555" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="558" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="557" t="n">
+        <v>20570</v>
       </c>
       <c r="G7" s="160" t="n"/>
     </row>
     <row r="8" ht="28.9" customHeight="1">
-      <c r="A8" s="60" t="n"/>
-      <c r="B8" s="331" t="n"/>
-      <c r="C8" s="539" t="n"/>
-      <c r="D8" s="540" t="n"/>
-      <c r="E8" s="516" t="n"/>
-      <c r="F8" s="542" t="n"/>
+      <c r="A8" s="60" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="331" t="inlineStr">
+        <is>
+          <t>VO6 - Wet Fire Sprinkler Upgrade to Ground Floor</t>
+        </is>
+      </c>
+      <c r="C8" s="554" t="n">
+        <v>32645.8</v>
+      </c>
+      <c r="D8" s="558" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="555" t="n">
+        <v>36154.8</v>
+      </c>
+      <c r="F8" s="559" t="n">
+        <v>0</v>
+      </c>
       <c r="G8" s="184" t="n"/>
     </row>
     <row r="9" ht="28.9" customHeight="1">
       <c r="A9" s="60" t="n"/>
-      <c r="B9" s="331" t="n"/>
-      <c r="C9" s="539" t="n"/>
-      <c r="D9" s="516" t="n"/>
-      <c r="E9" s="540" t="n"/>
-      <c r="F9" s="214" t="n"/>
+      <c r="B9" s="331" t="inlineStr">
+        <is>
+          <t>TOTALS</t>
+        </is>
+      </c>
+      <c r="C9" s="539">
+        <f>SUM(C4:C8)</f>
+        <v/>
+      </c>
+      <c r="D9" s="516">
+        <f>SUM(D4:D8)</f>
+        <v/>
+      </c>
+      <c r="E9" s="540">
+        <f>SUM(E4:E8)</f>
+        <v/>
+      </c>
+      <c r="F9" s="214">
+        <f>SUM(F4:F8)</f>
+        <v/>
+      </c>
       <c r="G9" s="160" t="n"/>
     </row>
     <row r="10" ht="28.9" customHeight="1">

</xml_diff>